<commit_message>
Features: Se asigna automaticamente una clave
</commit_message>
<xml_diff>
--- a/app/features/filleo/templates/formato-envio.xlsx
+++ b/app/features/filleo/templates/formato-envio.xlsx
@@ -526,7 +526,7 @@
         <v>70951063</v>
       </c>
       <c r="B2" s="3" t="n">
-        <v>921584492</v>
+        <v>987654321</v>
       </c>
       <c r="C2" s="3" t="n"/>
       <c r="D2" s="3" t="n"/>
@@ -538,7 +538,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>CERRO DE PASCO</t>
+          <t>ICA SAN JOAQUIN</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">

</xml_diff>